<commit_message>
add partial transform to DBF
</commit_message>
<xml_diff>
--- a/src/assets/schema/db_schema.xlsx
+++ b/src/assets/schema/db_schema.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Мои документы\Стас\Учеба\Проект_таксационных_карт\FGIS-LES\src\assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Мои документы\Стас\Учеба\Проект_таксационных_карт\FGIS-LES\src\assets\schema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40636B38-9784-4953-BA5D-F26DA7C24C65}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A88C79A0-5B7F-41AC-BDA8-B04A93D1BA20}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12600" xr2:uid="{AE1DFABD-FAB4-4AF3-B4B6-7526884842BF}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="268">
   <si>
     <t>Имя поля</t>
   </si>
@@ -36,9 +36,6 @@
     <t>MUK</t>
   </si>
   <si>
-    <t>Decimal (8,0)</t>
-  </si>
-  <si>
     <t>SRI</t>
   </si>
   <si>
@@ -822,9 +819,6 @@
     <t>KL</t>
   </si>
   <si>
-    <t>Char (35)</t>
-  </si>
-  <si>
     <t>№</t>
   </si>
   <si>
@@ -832,6 +826,9 @@
   </si>
   <si>
     <t>Char (13)</t>
+  </si>
+  <si>
+    <t>Char (70)</t>
   </si>
 </sst>
 </file>
@@ -1293,7 +1290,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1303,7 +1300,7 @@
       </c>
       <c r="D1" s="3"/>
     </row>
-    <row r="2" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -1311,7 +1308,7 @@
         <v>2</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" t="str">
@@ -1324,10 +1321,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>4</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>5</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" t="str">
@@ -1340,10 +1337,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" t="str">
@@ -1356,10 +1353,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" t="str">
@@ -1372,10 +1369,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>8</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>9</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" t="str">
@@ -1388,10 +1385,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" t="str">
@@ -1404,10 +1401,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>11</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>12</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" t="str">
@@ -1420,10 +1417,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>13</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>14</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" t="str">
@@ -1436,10 +1433,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" t="str">
@@ -1452,10 +1449,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>16</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>17</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" t="str">
@@ -1468,10 +1465,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" t="str">
@@ -1484,10 +1481,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D13" s="3"/>
       <c r="E13" t="str">
@@ -1500,10 +1497,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D14" s="3"/>
       <c r="E14" t="str">
@@ -1516,10 +1513,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D15" s="3"/>
       <c r="E15" t="str">
@@ -1532,10 +1529,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D16" s="3"/>
       <c r="E16" t="str">
@@ -1548,10 +1545,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="D17" s="3"/>
       <c r="E17" t="str">
@@ -1564,10 +1561,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D18" s="3"/>
       <c r="E18" t="str">
@@ -1580,10 +1577,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D19" s="3"/>
       <c r="E19" t="str">
@@ -1596,10 +1593,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D20" s="3"/>
       <c r="E20" t="str">
@@ -1612,10 +1609,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D21" s="3"/>
       <c r="E21" t="str">
@@ -1628,10 +1625,10 @@
         <v>21</v>
       </c>
       <c r="B22" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="D22" s="3"/>
       <c r="E22" t="str">
@@ -1644,10 +1641,10 @@
         <v>22</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D23" s="3"/>
       <c r="E23" t="str">
@@ -1660,10 +1657,10 @@
         <v>23</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D24" s="3"/>
       <c r="E24" t="str">
@@ -1676,10 +1673,10 @@
         <v>24</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D25" s="3"/>
       <c r="E25" t="str">
@@ -1692,10 +1689,10 @@
         <v>25</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D26" s="3"/>
       <c r="E26" t="str">
@@ -1708,10 +1705,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D27" s="3"/>
       <c r="E27" t="str">
@@ -1724,10 +1721,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D28" s="3"/>
       <c r="E28" t="str">
@@ -1740,10 +1737,10 @@
         <v>28</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D29" s="3"/>
       <c r="E29" t="str">
@@ -1756,10 +1753,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D30" s="3"/>
       <c r="E30" t="str">
@@ -1772,10 +1769,10 @@
         <v>30</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D31" s="3"/>
       <c r="E31" t="str">
@@ -1788,10 +1785,10 @@
         <v>31</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D32" s="3"/>
       <c r="E32" t="str">
@@ -1804,10 +1801,10 @@
         <v>32</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D33" s="3"/>
       <c r="E33" t="str">
@@ -1820,10 +1817,10 @@
         <v>33</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D34" s="3"/>
       <c r="E34" t="str">
@@ -1836,10 +1833,10 @@
         <v>34</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D35" s="3"/>
       <c r="E35" t="str">
@@ -1852,10 +1849,10 @@
         <v>35</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D36" s="3"/>
       <c r="E36" t="str">
@@ -1868,10 +1865,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D37" s="3"/>
       <c r="E37" t="str">
@@ -1884,10 +1881,10 @@
         <v>37</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D38" s="3"/>
       <c r="E38" t="str">
@@ -1900,10 +1897,10 @@
         <v>38</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D39" s="3"/>
       <c r="E39" t="str">
@@ -1916,10 +1913,10 @@
         <v>39</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D40" s="3"/>
       <c r="E40" t="str">
@@ -1932,10 +1929,10 @@
         <v>40</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D41" s="3"/>
       <c r="E41" t="str">
@@ -1948,10 +1945,10 @@
         <v>41</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D42" s="3"/>
       <c r="E42" t="str">
@@ -1964,10 +1961,10 @@
         <v>42</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D43" s="3"/>
       <c r="E43" t="str">
@@ -1980,10 +1977,10 @@
         <v>43</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D44" s="3"/>
       <c r="E44" t="str">
@@ -1996,10 +1993,10 @@
         <v>44</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D45" s="3"/>
       <c r="E45" t="str">
@@ -2012,10 +2009,10 @@
         <v>45</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D46" s="3"/>
       <c r="E46" t="str">
@@ -2028,10 +2025,10 @@
         <v>46</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D47" s="3"/>
       <c r="E47" t="str">
@@ -2044,10 +2041,10 @@
         <v>47</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D48" s="3"/>
       <c r="E48" t="str">
@@ -2060,10 +2057,10 @@
         <v>48</v>
       </c>
       <c r="B49" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C49" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="C49" s="5" t="s">
-        <v>60</v>
       </c>
       <c r="D49" s="3"/>
       <c r="E49" t="str">
@@ -2076,10 +2073,10 @@
         <v>49</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D50" s="3"/>
       <c r="E50" t="str">
@@ -2092,10 +2089,10 @@
         <v>50</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D51" s="3"/>
       <c r="E51" t="str">
@@ -2108,10 +2105,10 @@
         <v>51</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D52" s="3"/>
       <c r="E52" t="str">
@@ -2124,10 +2121,10 @@
         <v>52</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D53" s="6"/>
       <c r="E53" t="str">
@@ -2140,10 +2137,10 @@
         <v>53</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D54" s="3"/>
       <c r="E54" t="str">
@@ -2156,10 +2153,10 @@
         <v>54</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D55" s="3"/>
       <c r="E55" t="str">
@@ -2172,10 +2169,10 @@
         <v>55</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D56" s="3"/>
       <c r="E56" t="str">
@@ -2188,10 +2185,10 @@
         <v>56</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D57" s="3"/>
       <c r="E57" t="str">
@@ -2204,10 +2201,10 @@
         <v>57</v>
       </c>
       <c r="B58" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C58" s="5" t="s">
         <v>69</v>
-      </c>
-      <c r="C58" s="5" t="s">
-        <v>70</v>
       </c>
       <c r="D58" s="3"/>
       <c r="E58" t="str">
@@ -2220,10 +2217,10 @@
         <v>58</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D59" s="3"/>
       <c r="E59" t="str">
@@ -2236,10 +2233,10 @@
         <v>59</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D60" s="3"/>
       <c r="E60" t="str">
@@ -2252,10 +2249,10 @@
         <v>60</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D61" s="3"/>
       <c r="E61" t="str">
@@ -2268,10 +2265,10 @@
         <v>61</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D62" s="3"/>
       <c r="E62" t="str">
@@ -2284,10 +2281,10 @@
         <v>62</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D63" s="3"/>
       <c r="E63" t="str">
@@ -2300,10 +2297,10 @@
         <v>63</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D64" s="6"/>
       <c r="E64" t="str">
@@ -2316,10 +2313,10 @@
         <v>64</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D65" s="3"/>
       <c r="E65" t="str">
@@ -2332,10 +2329,10 @@
         <v>65</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D66" s="3"/>
       <c r="E66" t="str">
@@ -2348,10 +2345,10 @@
         <v>66</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D67" s="3"/>
       <c r="E67" t="str">
@@ -2364,10 +2361,10 @@
         <v>67</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D68" s="3"/>
       <c r="E68" t="str">
@@ -2380,10 +2377,10 @@
         <v>68</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D69" s="3"/>
       <c r="E69" t="str">
@@ -2396,10 +2393,10 @@
         <v>69</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D70" s="3"/>
       <c r="E70" t="str">
@@ -2412,10 +2409,10 @@
         <v>70</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D71" s="3"/>
       <c r="E71" t="str">
@@ -2428,10 +2425,10 @@
         <v>71</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D72" s="3"/>
       <c r="E72" t="str">
@@ -2444,10 +2441,10 @@
         <v>72</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D73" s="3"/>
       <c r="E73" t="str">
@@ -2460,10 +2457,10 @@
         <v>73</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D74" s="3"/>
       <c r="E74" t="str">
@@ -2476,10 +2473,10 @@
         <v>74</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D75" s="6"/>
       <c r="E75" t="str">
@@ -2492,10 +2489,10 @@
         <v>75</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D76" s="3"/>
       <c r="E76" t="str">
@@ -2508,10 +2505,10 @@
         <v>76</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D77" s="3"/>
       <c r="E77" t="str">
@@ -2524,10 +2521,10 @@
         <v>77</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D78" s="3"/>
       <c r="E78" t="str">
@@ -2540,10 +2537,10 @@
         <v>78</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D79" s="3"/>
       <c r="E79" t="str">
@@ -2556,10 +2553,10 @@
         <v>79</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D80" s="3"/>
       <c r="E80" t="str">
@@ -2572,10 +2569,10 @@
         <v>80</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D81" s="3"/>
       <c r="E81" t="str">
@@ -2588,10 +2585,10 @@
         <v>81</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D82" s="3"/>
       <c r="E82" t="str">
@@ -2604,10 +2601,10 @@
         <v>82</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D83" s="3"/>
       <c r="E83" t="str">
@@ -2620,10 +2617,10 @@
         <v>83</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D84" s="3"/>
       <c r="E84" t="str">
@@ -2636,10 +2633,10 @@
         <v>84</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D85" s="3"/>
       <c r="E85" t="str">
@@ -2652,10 +2649,10 @@
         <v>85</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D86" s="6"/>
       <c r="E86" t="str">
@@ -2668,10 +2665,10 @@
         <v>86</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D87" s="3"/>
       <c r="E87" t="str">
@@ -2684,10 +2681,10 @@
         <v>87</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D88" s="3"/>
       <c r="E88" t="str">
@@ -2700,10 +2697,10 @@
         <v>88</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C89" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D89" s="3"/>
       <c r="E89" t="str">
@@ -2716,10 +2713,10 @@
         <v>89</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D90" s="3"/>
       <c r="E90" t="str">
@@ -2732,10 +2729,10 @@
         <v>90</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D91" s="3"/>
       <c r="E91" t="str">
@@ -2748,10 +2745,10 @@
         <v>91</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D92" s="3"/>
       <c r="E92" t="str">
@@ -2764,10 +2761,10 @@
         <v>92</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D93" s="3"/>
       <c r="E93" t="str">
@@ -2780,10 +2777,10 @@
         <v>93</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C94" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D94" s="3"/>
       <c r="E94" t="str">
@@ -2796,10 +2793,10 @@
         <v>94</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C95" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D95" s="3"/>
       <c r="E95" t="str">
@@ -2812,10 +2809,10 @@
         <v>95</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C96" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D96" s="3"/>
       <c r="E96" t="str">
@@ -2828,10 +2825,10 @@
         <v>96</v>
       </c>
       <c r="B97" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C97" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D97" s="6"/>
       <c r="E97" t="str">
@@ -2844,10 +2841,10 @@
         <v>97</v>
       </c>
       <c r="B98" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C98" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D98" s="3"/>
       <c r="E98" t="str">
@@ -2860,10 +2857,10 @@
         <v>98</v>
       </c>
       <c r="B99" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C99" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D99" s="3"/>
       <c r="E99" t="str">
@@ -2876,10 +2873,10 @@
         <v>99</v>
       </c>
       <c r="B100" s="5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C100" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D100" s="3"/>
       <c r="E100" t="str">
@@ -2892,10 +2889,10 @@
         <v>100</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C101" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D101" s="3"/>
       <c r="E101" t="str">
@@ -2908,10 +2905,10 @@
         <v>101</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D102" s="3"/>
       <c r="E102" t="str">
@@ -2924,10 +2921,10 @@
         <v>102</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C103" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D103" s="3"/>
       <c r="E103" t="str">
@@ -2940,10 +2937,10 @@
         <v>103</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C104" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D104" s="3"/>
       <c r="E104" t="str">
@@ -2956,10 +2953,10 @@
         <v>104</v>
       </c>
       <c r="B105" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C105" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D105" s="3"/>
       <c r="E105" t="str">
@@ -2972,10 +2969,10 @@
         <v>105</v>
       </c>
       <c r="B106" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C106" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D106" s="3"/>
       <c r="E106" t="str">
@@ -2988,10 +2985,10 @@
         <v>106</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C107" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D107" s="3"/>
       <c r="E107" t="str">
@@ -3004,10 +3001,10 @@
         <v>107</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C108" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D108" s="6"/>
       <c r="E108" t="str">
@@ -3020,10 +3017,10 @@
         <v>108</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C109" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D109" s="3"/>
       <c r="E109" t="str">
@@ -3036,10 +3033,10 @@
         <v>109</v>
       </c>
       <c r="B110" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C110" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D110" s="3"/>
       <c r="E110" t="str">
@@ -3052,10 +3049,10 @@
         <v>110</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C111" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D111" s="3"/>
       <c r="E111" t="str">
@@ -3068,10 +3065,10 @@
         <v>111</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C112" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D112" s="3"/>
       <c r="E112" t="str">
@@ -3084,10 +3081,10 @@
         <v>112</v>
       </c>
       <c r="B113" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C113" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D113" s="3"/>
       <c r="E113" t="str">
@@ -3100,10 +3097,10 @@
         <v>113</v>
       </c>
       <c r="B114" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C114" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D114" s="3"/>
       <c r="E114" t="str">
@@ -3116,10 +3113,10 @@
         <v>114</v>
       </c>
       <c r="B115" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C115" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D115" s="3"/>
       <c r="E115" t="str">
@@ -3132,10 +3129,10 @@
         <v>115</v>
       </c>
       <c r="B116" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C116" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D116" s="3"/>
       <c r="E116" t="str">
@@ -3148,10 +3145,10 @@
         <v>116</v>
       </c>
       <c r="B117" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C117" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D117" s="3"/>
       <c r="E117" t="str">
@@ -3164,10 +3161,10 @@
         <v>117</v>
       </c>
       <c r="B118" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C118" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D118" s="3"/>
       <c r="E118" t="str">
@@ -3180,10 +3177,10 @@
         <v>118</v>
       </c>
       <c r="B119" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C119" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D119" s="6"/>
       <c r="E119" t="str">
@@ -3196,10 +3193,10 @@
         <v>119</v>
       </c>
       <c r="B120" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C120" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D120" s="3"/>
       <c r="E120" t="str">
@@ -3212,10 +3209,10 @@
         <v>120</v>
       </c>
       <c r="B121" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C121" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D121" s="3"/>
       <c r="E121" t="str">
@@ -3228,10 +3225,10 @@
         <v>121</v>
       </c>
       <c r="B122" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C122" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D122" s="3"/>
       <c r="E122" t="str">
@@ -3244,10 +3241,10 @@
         <v>122</v>
       </c>
       <c r="B123" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C123" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D123" s="3"/>
       <c r="E123" t="str">
@@ -3260,10 +3257,10 @@
         <v>123</v>
       </c>
       <c r="B124" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C124" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D124" s="3"/>
       <c r="E124" t="str">
@@ -3276,10 +3273,10 @@
         <v>124</v>
       </c>
       <c r="B125" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C125" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D125" s="3"/>
       <c r="E125" t="str">
@@ -3292,10 +3289,10 @@
         <v>125</v>
       </c>
       <c r="B126" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C126" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D126" s="3"/>
       <c r="E126" t="str">
@@ -3308,10 +3305,10 @@
         <v>126</v>
       </c>
       <c r="B127" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C127" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D127" s="3"/>
       <c r="E127" t="str">
@@ -3324,10 +3321,10 @@
         <v>127</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C128" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D128" s="3"/>
       <c r="E128" t="str">
@@ -3340,10 +3337,10 @@
         <v>128</v>
       </c>
       <c r="B129" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C129" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D129" s="3"/>
       <c r="E129" t="str">
@@ -3356,10 +3353,10 @@
         <v>129</v>
       </c>
       <c r="B130" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C130" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D130" s="6"/>
       <c r="E130" t="str">
@@ -3372,10 +3369,10 @@
         <v>130</v>
       </c>
       <c r="B131" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C131" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D131" s="3"/>
       <c r="E131" t="str">
@@ -3388,10 +3385,10 @@
         <v>131</v>
       </c>
       <c r="B132" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C132" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D132" s="3"/>
       <c r="E132" t="str">
@@ -3404,10 +3401,10 @@
         <v>132</v>
       </c>
       <c r="B133" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C133" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D133" s="3"/>
       <c r="E133" t="str">
@@ -3420,10 +3417,10 @@
         <v>133</v>
       </c>
       <c r="B134" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C134" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D134" s="3"/>
       <c r="E134" t="str">
@@ -3436,10 +3433,10 @@
         <v>134</v>
       </c>
       <c r="B135" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C135" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D135" s="3"/>
       <c r="E135" t="str">
@@ -3452,10 +3449,10 @@
         <v>135</v>
       </c>
       <c r="B136" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C136" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D136" s="3"/>
       <c r="E136" t="str">
@@ -3468,10 +3465,10 @@
         <v>136</v>
       </c>
       <c r="B137" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C137" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D137" s="3"/>
       <c r="E137" t="str">
@@ -3484,10 +3481,10 @@
         <v>137</v>
       </c>
       <c r="B138" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C138" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D138" s="3"/>
       <c r="E138" t="str">
@@ -3500,10 +3497,10 @@
         <v>138</v>
       </c>
       <c r="B139" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C139" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D139" s="3"/>
       <c r="E139" t="str">
@@ -3516,10 +3513,10 @@
         <v>139</v>
       </c>
       <c r="B140" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C140" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D140" s="3"/>
       <c r="E140" t="str">
@@ -3532,10 +3529,10 @@
         <v>140</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C141" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D141" s="6"/>
       <c r="E141" t="str">
@@ -3548,10 +3545,10 @@
         <v>141</v>
       </c>
       <c r="B142" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C142" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D142" s="3"/>
       <c r="E142" t="str">
@@ -3564,10 +3561,10 @@
         <v>142</v>
       </c>
       <c r="B143" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C143" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D143" s="3"/>
       <c r="E143" t="str">
@@ -3580,10 +3577,10 @@
         <v>143</v>
       </c>
       <c r="B144" s="5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C144" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D144" s="3"/>
       <c r="E144" t="str">
@@ -3596,10 +3593,10 @@
         <v>144</v>
       </c>
       <c r="B145" s="5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C145" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D145" s="3"/>
       <c r="E145" t="str">
@@ -3612,10 +3609,10 @@
         <v>145</v>
       </c>
       <c r="B146" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C146" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D146" s="3"/>
       <c r="E146" t="str">
@@ -3628,10 +3625,10 @@
         <v>146</v>
       </c>
       <c r="B147" s="5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C147" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D147" s="3"/>
       <c r="E147" t="str">
@@ -3644,10 +3641,10 @@
         <v>147</v>
       </c>
       <c r="B148" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C148" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D148" s="3"/>
       <c r="E148" t="str">
@@ -3660,10 +3657,10 @@
         <v>148</v>
       </c>
       <c r="B149" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C149" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D149" s="3"/>
       <c r="E149" t="str">
@@ -3676,10 +3673,10 @@
         <v>149</v>
       </c>
       <c r="B150" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C150" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D150" s="3"/>
       <c r="E150" t="str">
@@ -3692,10 +3689,10 @@
         <v>150</v>
       </c>
       <c r="B151" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C151" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D151" s="3"/>
       <c r="E151" t="str">
@@ -3708,10 +3705,10 @@
         <v>151</v>
       </c>
       <c r="B152" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C152" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D152" s="6"/>
       <c r="E152" t="str">
@@ -3724,10 +3721,10 @@
         <v>152</v>
       </c>
       <c r="B153" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C153" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D153" s="3"/>
       <c r="E153" t="str">
@@ -3740,10 +3737,10 @@
         <v>153</v>
       </c>
       <c r="B154" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C154" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D154" s="3"/>
       <c r="E154" t="str">
@@ -3756,10 +3753,10 @@
         <v>154</v>
       </c>
       <c r="B155" s="5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C155" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D155" s="3"/>
       <c r="E155" t="str">
@@ -3772,10 +3769,10 @@
         <v>155</v>
       </c>
       <c r="B156" s="5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C156" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D156" s="3"/>
       <c r="E156" t="str">
@@ -3788,10 +3785,10 @@
         <v>156</v>
       </c>
       <c r="B157" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C157" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D157" s="3"/>
       <c r="E157" t="str">
@@ -3804,10 +3801,10 @@
         <v>157</v>
       </c>
       <c r="B158" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C158" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D158" s="3"/>
       <c r="E158" t="str">
@@ -3820,10 +3817,10 @@
         <v>158</v>
       </c>
       <c r="B159" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C159" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D159" s="3"/>
       <c r="E159" t="str">
@@ -3836,10 +3833,10 @@
         <v>159</v>
       </c>
       <c r="B160" s="5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C160" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D160" s="3"/>
       <c r="E160" t="str">
@@ -3852,10 +3849,10 @@
         <v>160</v>
       </c>
       <c r="B161" s="5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C161" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D161" s="3"/>
       <c r="E161" t="str">
@@ -3868,10 +3865,10 @@
         <v>161</v>
       </c>
       <c r="B162" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C162" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D162" s="3"/>
       <c r="E162" t="str">
@@ -3884,10 +3881,10 @@
         <v>162</v>
       </c>
       <c r="B163" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C163" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D163" s="6"/>
       <c r="E163" t="str">
@@ -3900,10 +3897,10 @@
         <v>163</v>
       </c>
       <c r="B164" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="C164" s="5" t="s">
         <v>176</v>
-      </c>
-      <c r="C164" s="5" t="s">
-        <v>177</v>
       </c>
       <c r="D164" s="3"/>
       <c r="E164" t="str">
@@ -3916,10 +3913,10 @@
         <v>164</v>
       </c>
       <c r="B165" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C165" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D165" s="3"/>
       <c r="E165" t="str">
@@ -3932,10 +3929,10 @@
         <v>165</v>
       </c>
       <c r="B166" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C166" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D166" s="3"/>
       <c r="E166" t="str">
@@ -3948,10 +3945,10 @@
         <v>166</v>
       </c>
       <c r="B167" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C167" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D167" s="3"/>
       <c r="E167" t="str">
@@ -3964,10 +3961,10 @@
         <v>167</v>
       </c>
       <c r="B168" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C168" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D168" s="3"/>
       <c r="E168" t="str">
@@ -3980,10 +3977,10 @@
         <v>168</v>
       </c>
       <c r="B169" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C169" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D169" s="3"/>
       <c r="E169" t="str">
@@ -3996,10 +3993,10 @@
         <v>169</v>
       </c>
       <c r="B170" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C170" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D170" s="3"/>
       <c r="E170" t="str">
@@ -4012,10 +4009,10 @@
         <v>170</v>
       </c>
       <c r="B171" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C171" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D171" s="3"/>
       <c r="E171" t="str">
@@ -4028,10 +4025,10 @@
         <v>171</v>
       </c>
       <c r="B172" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C172" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D172" s="3"/>
       <c r="E172" t="str">
@@ -4044,10 +4041,10 @@
         <v>172</v>
       </c>
       <c r="B173" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C173" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D173" s="6"/>
       <c r="E173" t="str">
@@ -4060,10 +4057,10 @@
         <v>173</v>
       </c>
       <c r="B174" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C174" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D174" s="3"/>
       <c r="E174" t="str">
@@ -4076,10 +4073,10 @@
         <v>174</v>
       </c>
       <c r="B175" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C175" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D175" s="3"/>
       <c r="E175" t="str">
@@ -4092,10 +4089,10 @@
         <v>175</v>
       </c>
       <c r="B176" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C176" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D176" s="3"/>
       <c r="E176" t="str">
@@ -4108,10 +4105,10 @@
         <v>176</v>
       </c>
       <c r="B177" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C177" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D177" s="6"/>
       <c r="E177" t="str">
@@ -4124,10 +4121,10 @@
         <v>177</v>
       </c>
       <c r="B178" s="5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C178" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D178" s="3"/>
       <c r="E178" t="str">
@@ -4140,10 +4137,10 @@
         <v>178</v>
       </c>
       <c r="B179" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="C179" s="5" t="s">
         <v>192</v>
-      </c>
-      <c r="C179" s="5" t="s">
-        <v>193</v>
       </c>
       <c r="D179" s="3"/>
       <c r="E179" t="str">
@@ -4156,10 +4153,10 @@
         <v>179</v>
       </c>
       <c r="B180" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C180" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D180" s="3"/>
       <c r="E180" t="str">
@@ -4172,10 +4169,10 @@
         <v>180</v>
       </c>
       <c r="B181" s="5" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C181" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D181" s="3"/>
       <c r="E181" t="str">
@@ -4188,10 +4185,10 @@
         <v>181</v>
       </c>
       <c r="B182" s="5" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C182" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D182" s="3"/>
       <c r="E182" t="str">
@@ -4204,10 +4201,10 @@
         <v>182</v>
       </c>
       <c r="B183" s="5" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C183" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D183" s="3"/>
       <c r="E183" t="str">
@@ -4220,10 +4217,10 @@
         <v>183</v>
       </c>
       <c r="B184" s="5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C184" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D184" s="3"/>
       <c r="E184" t="str">
@@ -4236,10 +4233,10 @@
         <v>184</v>
       </c>
       <c r="B185" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C185" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D185" s="3"/>
       <c r="E185" t="str">
@@ -4252,10 +4249,10 @@
         <v>185</v>
       </c>
       <c r="B186" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C186" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D186" s="6"/>
       <c r="E186" t="str">
@@ -4268,10 +4265,10 @@
         <v>186</v>
       </c>
       <c r="B187" s="5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C187" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D187" s="3"/>
       <c r="E187" t="str">
@@ -4284,10 +4281,10 @@
         <v>187</v>
       </c>
       <c r="B188" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C188" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D188" s="3"/>
       <c r="E188" t="str">
@@ -4300,10 +4297,10 @@
         <v>188</v>
       </c>
       <c r="B189" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C189" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D189" s="3"/>
       <c r="E189" t="str">
@@ -4316,10 +4313,10 @@
         <v>189</v>
       </c>
       <c r="B190" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C190" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D190" s="3"/>
       <c r="E190" t="str">
@@ -4332,10 +4329,10 @@
         <v>190</v>
       </c>
       <c r="B191" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C191" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D191" s="3"/>
       <c r="E191" t="str">
@@ -4348,10 +4345,10 @@
         <v>191</v>
       </c>
       <c r="B192" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C192" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D192" s="3"/>
       <c r="E192" t="str">
@@ -4364,10 +4361,10 @@
         <v>192</v>
       </c>
       <c r="B193" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C193" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D193" s="3"/>
       <c r="E193" t="str">
@@ -4380,10 +4377,10 @@
         <v>193</v>
       </c>
       <c r="B194" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C194" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D194" s="3"/>
       <c r="E194" t="str">
@@ -4396,10 +4393,10 @@
         <v>194</v>
       </c>
       <c r="B195" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C195" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D195" s="6"/>
       <c r="E195" t="str">
@@ -4412,10 +4409,10 @@
         <v>195</v>
       </c>
       <c r="B196" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C196" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D196" s="3"/>
       <c r="E196" t="str">
@@ -4428,10 +4425,10 @@
         <v>196</v>
       </c>
       <c r="B197" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C197" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D197" s="3"/>
       <c r="E197" t="str">
@@ -4444,10 +4441,10 @@
         <v>197</v>
       </c>
       <c r="B198" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C198" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D198" s="3"/>
       <c r="E198" t="str">
@@ -4460,10 +4457,10 @@
         <v>198</v>
       </c>
       <c r="B199" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C199" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D199" s="3"/>
       <c r="E199" t="str">
@@ -4476,10 +4473,10 @@
         <v>199</v>
       </c>
       <c r="B200" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C200" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D200" s="3"/>
       <c r="E200" t="str">
@@ -4492,10 +4489,10 @@
         <v>200</v>
       </c>
       <c r="B201" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C201" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D201" s="3"/>
       <c r="E201" t="str">
@@ -4508,10 +4505,10 @@
         <v>201</v>
       </c>
       <c r="B202" s="5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C202" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D202" s="3"/>
       <c r="E202" t="str">
@@ -4524,10 +4521,10 @@
         <v>202</v>
       </c>
       <c r="B203" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C203" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D203" s="3"/>
       <c r="E203" t="str">
@@ -4540,10 +4537,10 @@
         <v>203</v>
       </c>
       <c r="B204" s="5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C204" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D204" s="6"/>
       <c r="E204" t="str">
@@ -4556,10 +4553,10 @@
         <v>204</v>
       </c>
       <c r="B205" s="5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C205" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D205" s="3"/>
       <c r="E205" t="str">
@@ -4572,10 +4569,10 @@
         <v>205</v>
       </c>
       <c r="B206" s="5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C206" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D206" s="3"/>
       <c r="E206" t="str">
@@ -4588,10 +4585,10 @@
         <v>206</v>
       </c>
       <c r="B207" s="5" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C207" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D207" s="3"/>
       <c r="E207" t="str">
@@ -4604,10 +4601,10 @@
         <v>207</v>
       </c>
       <c r="B208" s="5" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C208" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D208" s="3"/>
       <c r="E208" t="str">
@@ -4620,10 +4617,10 @@
         <v>208</v>
       </c>
       <c r="B209" s="5" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C209" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D209" s="3"/>
       <c r="E209" t="str">
@@ -4636,10 +4633,10 @@
         <v>209</v>
       </c>
       <c r="B210" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C210" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D210" s="3"/>
       <c r="E210" t="str">
@@ -4652,10 +4649,10 @@
         <v>210</v>
       </c>
       <c r="B211" s="5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C211" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D211" s="3"/>
       <c r="E211" t="str">
@@ -4668,10 +4665,10 @@
         <v>211</v>
       </c>
       <c r="B212" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C212" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D212" s="3"/>
       <c r="E212" t="str">
@@ -4684,10 +4681,10 @@
         <v>212</v>
       </c>
       <c r="B213" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C213" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D213" s="6"/>
       <c r="E213" t="str">
@@ -4700,10 +4697,10 @@
         <v>213</v>
       </c>
       <c r="B214" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C214" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D214" s="3"/>
       <c r="E214" t="str">
@@ -4716,10 +4713,10 @@
         <v>214</v>
       </c>
       <c r="B215" s="5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C215" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D215" s="3"/>
       <c r="E215" t="str">
@@ -4732,10 +4729,10 @@
         <v>215</v>
       </c>
       <c r="B216" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C216" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D216" s="3"/>
       <c r="E216" t="str">
@@ -4748,10 +4745,10 @@
         <v>216</v>
       </c>
       <c r="B217" s="5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C217" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D217" s="3"/>
       <c r="E217" t="str">
@@ -4764,10 +4761,10 @@
         <v>217</v>
       </c>
       <c r="B218" s="5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C218" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D218" s="3"/>
       <c r="E218" t="str">
@@ -4780,10 +4777,10 @@
         <v>218</v>
       </c>
       <c r="B219" s="5" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C219" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D219" s="3"/>
       <c r="E219" t="str">
@@ -4796,10 +4793,10 @@
         <v>219</v>
       </c>
       <c r="B220" s="5" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C220" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D220" s="3"/>
       <c r="E220" t="str">
@@ -4812,10 +4809,10 @@
         <v>220</v>
       </c>
       <c r="B221" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C221" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D221" s="3"/>
       <c r="E221" t="str">
@@ -4828,10 +4825,10 @@
         <v>221</v>
       </c>
       <c r="B222" s="5" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C222" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D222" s="6"/>
       <c r="E222" t="str">
@@ -4844,10 +4841,10 @@
         <v>222</v>
       </c>
       <c r="B223" s="5" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C223" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D223" s="3"/>
       <c r="E223" t="str">
@@ -4860,10 +4857,10 @@
         <v>223</v>
       </c>
       <c r="B224" s="5" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C224" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D224" s="3"/>
       <c r="E224" t="str">
@@ -4876,10 +4873,10 @@
         <v>224</v>
       </c>
       <c r="B225" s="5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C225" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D225" s="3"/>
       <c r="E225" t="str">
@@ -4892,10 +4889,10 @@
         <v>225</v>
       </c>
       <c r="B226" s="5" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C226" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D226" s="3"/>
       <c r="E226" t="str">
@@ -4908,10 +4905,10 @@
         <v>226</v>
       </c>
       <c r="B227" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C227" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D227" s="3"/>
       <c r="E227" t="str">
@@ -4924,10 +4921,10 @@
         <v>227</v>
       </c>
       <c r="B228" s="5" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C228" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D228" s="3"/>
       <c r="E228" t="str">
@@ -4940,10 +4937,10 @@
         <v>228</v>
       </c>
       <c r="B229" s="5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C229" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D229" s="3"/>
       <c r="E229" t="str">
@@ -4956,10 +4953,10 @@
         <v>229</v>
       </c>
       <c r="B230" s="5" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C230" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D230" s="3"/>
       <c r="E230" t="str">
@@ -4972,10 +4969,10 @@
         <v>230</v>
       </c>
       <c r="B231" s="5" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C231" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D231" s="6"/>
       <c r="E231" t="str">
@@ -4988,10 +4985,10 @@
         <v>231</v>
       </c>
       <c r="B232" s="5" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C232" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D232" s="3"/>
       <c r="E232" t="str">
@@ -5004,10 +5001,10 @@
         <v>232</v>
       </c>
       <c r="B233" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C233" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D233" s="3"/>
       <c r="E233" t="str">
@@ -5020,10 +5017,10 @@
         <v>233</v>
       </c>
       <c r="B234" s="5" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C234" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D234" s="3"/>
       <c r="E234" t="str">
@@ -5036,10 +5033,10 @@
         <v>234</v>
       </c>
       <c r="B235" s="5" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C235" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D235" s="3"/>
       <c r="E235" t="str">
@@ -5052,10 +5049,10 @@
         <v>235</v>
       </c>
       <c r="B236" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C236" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D236" s="3"/>
       <c r="E236" t="str">
@@ -5068,10 +5065,10 @@
         <v>236</v>
       </c>
       <c r="B237" s="5" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C237" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D237" s="3"/>
       <c r="E237" t="str">
@@ -5084,10 +5081,10 @@
         <v>237</v>
       </c>
       <c r="B238" s="5" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C238" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D238" s="3"/>
       <c r="E238" t="str">
@@ -5100,10 +5097,10 @@
         <v>238</v>
       </c>
       <c r="B239" s="5" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C239" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D239" s="3"/>
       <c r="E239" t="str">
@@ -5116,10 +5113,10 @@
         <v>239</v>
       </c>
       <c r="B240" s="5" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C240" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D240" s="6"/>
       <c r="E240" t="str">
@@ -5132,10 +5129,10 @@
         <v>240</v>
       </c>
       <c r="B241" s="5" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C241" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D241" s="3"/>
       <c r="E241" t="str">
@@ -5148,10 +5145,10 @@
         <v>241</v>
       </c>
       <c r="B242" s="5" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C242" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D242" s="3"/>
       <c r="E242" t="str">
@@ -5164,10 +5161,10 @@
         <v>242</v>
       </c>
       <c r="B243" s="5" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C243" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D243" s="3"/>
       <c r="E243" t="str">
@@ -5180,10 +5177,10 @@
         <v>243</v>
       </c>
       <c r="B244" s="5" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C244" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D244" s="3"/>
       <c r="E244" t="str">
@@ -5196,10 +5193,10 @@
         <v>244</v>
       </c>
       <c r="B245" s="5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C245" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D245" s="3"/>
       <c r="E245" t="str">
@@ -5212,10 +5209,10 @@
         <v>245</v>
       </c>
       <c r="B246" s="5" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C246" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D246" s="3"/>
       <c r="E246" t="str">
@@ -5228,10 +5225,10 @@
         <v>246</v>
       </c>
       <c r="B247" s="5" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C247" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D247" s="3"/>
       <c r="E247" t="str">
@@ -5244,10 +5241,10 @@
         <v>247</v>
       </c>
       <c r="B248" s="5" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C248" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D248" s="3"/>
       <c r="E248" t="str">
@@ -5260,10 +5257,10 @@
         <v>248</v>
       </c>
       <c r="B249" s="5" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C249" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D249" s="3"/>
       <c r="E249" t="str">
@@ -5276,10 +5273,10 @@
         <v>249</v>
       </c>
       <c r="B250" s="5" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C250" s="5" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D250" s="3"/>
       <c r="E250" t="str">
@@ -5292,10 +5289,10 @@
         <v>250</v>
       </c>
       <c r="B251" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="C251" s="5" t="s">
         <v>267</v>
-      </c>
-      <c r="C251" s="5" t="s">
-        <v>265</v>
       </c>
       <c r="D251" s="3"/>
       <c r="E251" t="str">

</xml_diff>

<commit_message>
hot fix to fgis-les
</commit_message>
<xml_diff>
--- a/src/assets/schema/db_schema.xlsx
+++ b/src/assets/schema/db_schema.xlsx
@@ -1,23 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23426"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Мои документы\Стас\Учеба\Проект_таксационных_карт\FGIS-LES\src\assets\schema\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A88C79A0-5B7F-41AC-BDA8-B04A93D1BA20}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="7" rupBuild="4507"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12600" xr2:uid="{AE1DFABD-FAB4-4AF3-B4B6-7526884842BF}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12600"/>
   </bookViews>
   <sheets>
     <sheet name="schema" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+  <calcPr calcId="125725"/>
+  <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -828,14 +822,14 @@
     <t>Char (13)</t>
   </si>
   <si>
-    <t>Char (70)</t>
+    <t>Char (50)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1028,7 +1022,7 @@
     </a:clrScheme>
     <a:fontScheme name="Стандартная">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -1080,7 +1074,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -1274,21 +1268,21 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1494EC8E-07DF-410B-9371-E993052E9DA8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E251"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="3" width="15.6640625" customWidth="1"/>
+    <col min="1" max="3" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="16.5" thickBot="1">
       <c r="A1" s="1" t="s">
         <v>264</v>
       </c>
@@ -1300,7 +1294,7 @@
       </c>
       <c r="D1" s="3"/>
     </row>
-    <row r="2" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" ht="16.5" thickBot="1">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -1316,7 +1310,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" ht="16.5" thickBot="1">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -1332,7 +1326,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="16.5" thickBot="1">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -1348,7 +1342,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" ht="16.5" thickBot="1">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -1364,7 +1358,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="16.5" thickBot="1">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -1380,7 +1374,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" ht="16.5" thickBot="1">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -1396,7 +1390,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="16.5" thickBot="1">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -1412,7 +1406,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="16.5" thickBot="1">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -1428,7 +1422,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" ht="16.5" thickBot="1">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -1444,7 +1438,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" ht="16.5" thickBot="1">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -1460,7 +1454,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" ht="16.5" thickBot="1">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -1476,7 +1470,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" ht="16.5" thickBot="1">
       <c r="A13" s="4">
         <v>12</v>
       </c>
@@ -1492,7 +1486,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" ht="16.5" thickBot="1">
       <c r="A14" s="4">
         <v>13</v>
       </c>
@@ -1508,7 +1502,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" ht="16.5" thickBot="1">
       <c r="A15" s="4">
         <v>14</v>
       </c>
@@ -1524,7 +1518,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" ht="16.5" thickBot="1">
       <c r="A16" s="4">
         <v>15</v>
       </c>
@@ -1540,7 +1534,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" ht="16.5" thickBot="1">
       <c r="A17" s="4">
         <v>16</v>
       </c>
@@ -1556,7 +1550,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" ht="16.5" thickBot="1">
       <c r="A18" s="4">
         <v>17</v>
       </c>
@@ -1572,7 +1566,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" ht="16.5" thickBot="1">
       <c r="A19" s="4">
         <v>18</v>
       </c>
@@ -1588,7 +1582,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" ht="16.5" thickBot="1">
       <c r="A20" s="4">
         <v>19</v>
       </c>
@@ -1604,7 +1598,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" ht="16.5" thickBot="1">
       <c r="A21" s="4">
         <v>20</v>
       </c>
@@ -1620,7 +1614,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" ht="16.5" thickBot="1">
       <c r="A22" s="4">
         <v>21</v>
       </c>
@@ -1636,7 +1630,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" ht="16.5" thickBot="1">
       <c r="A23" s="4">
         <v>22</v>
       </c>
@@ -1652,7 +1646,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" ht="16.5" thickBot="1">
       <c r="A24" s="4">
         <v>23</v>
       </c>
@@ -1668,7 +1662,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" ht="16.5" thickBot="1">
       <c r="A25" s="4">
         <v>24</v>
       </c>
@@ -1684,7 +1678,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" ht="16.5" thickBot="1">
       <c r="A26" s="4">
         <v>25</v>
       </c>
@@ -1700,7 +1694,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" ht="16.5" thickBot="1">
       <c r="A27" s="4">
         <v>26</v>
       </c>
@@ -1716,7 +1710,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" ht="16.5" thickBot="1">
       <c r="A28" s="4">
         <v>27</v>
       </c>
@@ -1732,7 +1726,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" ht="16.5" thickBot="1">
       <c r="A29" s="4">
         <v>28</v>
       </c>
@@ -1748,7 +1742,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" ht="16.5" thickBot="1">
       <c r="A30" s="4">
         <v>29</v>
       </c>
@@ -1764,7 +1758,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" ht="16.5" thickBot="1">
       <c r="A31" s="4">
         <v>30</v>
       </c>
@@ -1780,7 +1774,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" ht="16.5" thickBot="1">
       <c r="A32" s="4">
         <v>31</v>
       </c>
@@ -1796,7 +1790,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" ht="16.5" thickBot="1">
       <c r="A33" s="4">
         <v>32</v>
       </c>
@@ -1812,7 +1806,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" ht="16.5" thickBot="1">
       <c r="A34" s="4">
         <v>33</v>
       </c>
@@ -1828,7 +1822,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" ht="16.5" thickBot="1">
       <c r="A35" s="4">
         <v>34</v>
       </c>
@@ -1844,7 +1838,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" ht="16.5" thickBot="1">
       <c r="A36" s="4">
         <v>35</v>
       </c>
@@ -1860,7 +1854,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" ht="16.5" thickBot="1">
       <c r="A37" s="4">
         <v>36</v>
       </c>
@@ -1876,7 +1870,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" ht="16.5" thickBot="1">
       <c r="A38" s="4">
         <v>37</v>
       </c>
@@ -1892,7 +1886,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" ht="16.5" thickBot="1">
       <c r="A39" s="4">
         <v>38</v>
       </c>
@@ -1908,7 +1902,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" ht="16.5" thickBot="1">
       <c r="A40" s="4">
         <v>39</v>
       </c>
@@ -1924,7 +1918,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" ht="16.5" thickBot="1">
       <c r="A41" s="4">
         <v>40</v>
       </c>
@@ -1940,7 +1934,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" ht="16.5" thickBot="1">
       <c r="A42" s="4">
         <v>41</v>
       </c>
@@ -1956,7 +1950,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" ht="16.5" thickBot="1">
       <c r="A43" s="4">
         <v>42</v>
       </c>
@@ -1972,7 +1966,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" ht="16.5" thickBot="1">
       <c r="A44" s="4">
         <v>43</v>
       </c>
@@ -1988,7 +1982,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" ht="16.5" thickBot="1">
       <c r="A45" s="4">
         <v>44</v>
       </c>
@@ -2004,7 +1998,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="46" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" ht="16.5" thickBot="1">
       <c r="A46" s="4">
         <v>45</v>
       </c>
@@ -2020,7 +2014,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" ht="16.5" thickBot="1">
       <c r="A47" s="4">
         <v>46</v>
       </c>
@@ -2036,7 +2030,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" ht="16.5" thickBot="1">
       <c r="A48" s="4">
         <v>47</v>
       </c>
@@ -2052,7 +2046,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" ht="16.5" thickBot="1">
       <c r="A49" s="4">
         <v>48</v>
       </c>
@@ -2068,7 +2062,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" ht="16.5" thickBot="1">
       <c r="A50" s="4">
         <v>49</v>
       </c>
@@ -2084,7 +2078,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" ht="16.5" thickBot="1">
       <c r="A51" s="4">
         <v>50</v>
       </c>
@@ -2100,7 +2094,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" ht="16.5" thickBot="1">
       <c r="A52" s="4">
         <v>51</v>
       </c>
@@ -2116,7 +2110,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" ht="16.5" thickBot="1">
       <c r="A53" s="4">
         <v>52</v>
       </c>
@@ -2132,7 +2126,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" ht="16.5" thickBot="1">
       <c r="A54" s="4">
         <v>53</v>
       </c>
@@ -2148,7 +2142,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" ht="16.5" thickBot="1">
       <c r="A55" s="4">
         <v>54</v>
       </c>
@@ -2164,7 +2158,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" ht="16.5" thickBot="1">
       <c r="A56" s="4">
         <v>55</v>
       </c>
@@ -2180,7 +2174,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" ht="16.5" thickBot="1">
       <c r="A57" s="4">
         <v>56</v>
       </c>
@@ -2196,7 +2190,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" ht="16.5" thickBot="1">
       <c r="A58" s="4">
         <v>57</v>
       </c>
@@ -2212,7 +2206,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" ht="16.5" thickBot="1">
       <c r="A59" s="4">
         <v>58</v>
       </c>
@@ -2228,7 +2222,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="60" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" ht="16.5" thickBot="1">
       <c r="A60" s="4">
         <v>59</v>
       </c>
@@ -2244,7 +2238,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="61" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" ht="16.5" thickBot="1">
       <c r="A61" s="4">
         <v>60</v>
       </c>
@@ -2260,7 +2254,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="62" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" ht="16.5" thickBot="1">
       <c r="A62" s="4">
         <v>61</v>
       </c>
@@ -2276,7 +2270,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="63" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" ht="16.5" thickBot="1">
       <c r="A63" s="4">
         <v>62</v>
       </c>
@@ -2292,7 +2286,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="64" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" ht="16.5" thickBot="1">
       <c r="A64" s="4">
         <v>63</v>
       </c>
@@ -2308,7 +2302,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="65" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" ht="16.5" thickBot="1">
       <c r="A65" s="4">
         <v>64</v>
       </c>
@@ -2324,7 +2318,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="66" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" ht="16.5" thickBot="1">
       <c r="A66" s="4">
         <v>65</v>
       </c>
@@ -2340,7 +2334,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="67" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" ht="16.5" thickBot="1">
       <c r="A67" s="4">
         <v>66</v>
       </c>
@@ -2356,7 +2350,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="68" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" ht="16.5" thickBot="1">
       <c r="A68" s="4">
         <v>67</v>
       </c>
@@ -2372,7 +2366,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="69" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" ht="16.5" thickBot="1">
       <c r="A69" s="4">
         <v>68</v>
       </c>
@@ -2388,7 +2382,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="70" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" ht="16.5" thickBot="1">
       <c r="A70" s="4">
         <v>69</v>
       </c>
@@ -2404,7 +2398,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="71" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" ht="16.5" thickBot="1">
       <c r="A71" s="4">
         <v>70</v>
       </c>
@@ -2420,7 +2414,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="72" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" ht="16.5" thickBot="1">
       <c r="A72" s="4">
         <v>71</v>
       </c>
@@ -2436,7 +2430,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="73" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" ht="16.5" thickBot="1">
       <c r="A73" s="4">
         <v>72</v>
       </c>
@@ -2452,7 +2446,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="74" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" ht="16.5" thickBot="1">
       <c r="A74" s="4">
         <v>73</v>
       </c>
@@ -2468,7 +2462,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="75" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" ht="16.5" thickBot="1">
       <c r="A75" s="4">
         <v>74</v>
       </c>
@@ -2484,7 +2478,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="76" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" ht="16.5" thickBot="1">
       <c r="A76" s="4">
         <v>75</v>
       </c>
@@ -2500,7 +2494,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="77" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" ht="16.5" thickBot="1">
       <c r="A77" s="4">
         <v>76</v>
       </c>
@@ -2516,7 +2510,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="78" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" ht="16.5" thickBot="1">
       <c r="A78" s="4">
         <v>77</v>
       </c>
@@ -2532,7 +2526,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="79" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" ht="16.5" thickBot="1">
       <c r="A79" s="4">
         <v>78</v>
       </c>
@@ -2548,7 +2542,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="80" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" ht="16.5" thickBot="1">
       <c r="A80" s="4">
         <v>79</v>
       </c>
@@ -2564,7 +2558,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="81" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" ht="16.5" thickBot="1">
       <c r="A81" s="4">
         <v>80</v>
       </c>
@@ -2580,7 +2574,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="82" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" ht="16.5" thickBot="1">
       <c r="A82" s="4">
         <v>81</v>
       </c>
@@ -2596,7 +2590,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="83" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" ht="16.5" thickBot="1">
       <c r="A83" s="4">
         <v>82</v>
       </c>
@@ -2612,7 +2606,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="84" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" ht="16.5" thickBot="1">
       <c r="A84" s="4">
         <v>83</v>
       </c>
@@ -2628,7 +2622,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="85" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" ht="16.5" thickBot="1">
       <c r="A85" s="4">
         <v>84</v>
       </c>
@@ -2644,7 +2638,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="86" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" ht="16.5" thickBot="1">
       <c r="A86" s="4">
         <v>85</v>
       </c>
@@ -2660,7 +2654,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="87" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" ht="16.5" thickBot="1">
       <c r="A87" s="4">
         <v>86</v>
       </c>
@@ -2676,7 +2670,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="88" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" ht="16.5" thickBot="1">
       <c r="A88" s="4">
         <v>87</v>
       </c>
@@ -2692,7 +2686,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="89" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" ht="16.5" thickBot="1">
       <c r="A89" s="4">
         <v>88</v>
       </c>
@@ -2708,7 +2702,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="90" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" ht="16.5" thickBot="1">
       <c r="A90" s="4">
         <v>89</v>
       </c>
@@ -2724,7 +2718,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="91" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" ht="16.5" thickBot="1">
       <c r="A91" s="4">
         <v>90</v>
       </c>
@@ -2740,7 +2734,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="92" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" ht="16.5" thickBot="1">
       <c r="A92" s="4">
         <v>91</v>
       </c>
@@ -2756,7 +2750,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="93" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" ht="16.5" thickBot="1">
       <c r="A93" s="4">
         <v>92</v>
       </c>
@@ -2772,7 +2766,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="94" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" ht="16.5" thickBot="1">
       <c r="A94" s="4">
         <v>93</v>
       </c>
@@ -2788,7 +2782,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="95" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" ht="16.5" thickBot="1">
       <c r="A95" s="4">
         <v>94</v>
       </c>
@@ -2804,7 +2798,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="96" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" ht="16.5" thickBot="1">
       <c r="A96" s="4">
         <v>95</v>
       </c>
@@ -2820,7 +2814,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="97" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" ht="16.5" thickBot="1">
       <c r="A97" s="4">
         <v>96</v>
       </c>
@@ -2836,7 +2830,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="98" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" ht="16.5" thickBot="1">
       <c r="A98" s="4">
         <v>97</v>
       </c>
@@ -2852,7 +2846,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="99" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" ht="16.5" thickBot="1">
       <c r="A99" s="4">
         <v>98</v>
       </c>
@@ -2868,7 +2862,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="100" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" ht="16.5" thickBot="1">
       <c r="A100" s="4">
         <v>99</v>
       </c>
@@ -2884,7 +2878,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="101" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" ht="16.5" thickBot="1">
       <c r="A101" s="4">
         <v>100</v>
       </c>
@@ -2900,7 +2894,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="102" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" ht="16.5" thickBot="1">
       <c r="A102" s="4">
         <v>101</v>
       </c>
@@ -2916,7 +2910,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="103" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" ht="16.5" thickBot="1">
       <c r="A103" s="4">
         <v>102</v>
       </c>
@@ -2932,7 +2926,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="104" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" ht="16.5" thickBot="1">
       <c r="A104" s="4">
         <v>103</v>
       </c>
@@ -2948,7 +2942,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="105" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" ht="16.5" thickBot="1">
       <c r="A105" s="4">
         <v>104</v>
       </c>
@@ -2964,7 +2958,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="106" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" ht="16.5" thickBot="1">
       <c r="A106" s="4">
         <v>105</v>
       </c>
@@ -2980,7 +2974,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="107" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" ht="16.5" thickBot="1">
       <c r="A107" s="4">
         <v>106</v>
       </c>
@@ -2996,7 +2990,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="108" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" ht="16.5" thickBot="1">
       <c r="A108" s="4">
         <v>107</v>
       </c>
@@ -3012,7 +3006,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="109" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" ht="16.5" thickBot="1">
       <c r="A109" s="4">
         <v>108</v>
       </c>
@@ -3028,7 +3022,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="110" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" ht="16.5" thickBot="1">
       <c r="A110" s="4">
         <v>109</v>
       </c>
@@ -3044,7 +3038,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="111" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" ht="16.5" thickBot="1">
       <c r="A111" s="4">
         <v>110</v>
       </c>
@@ -3060,7 +3054,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="112" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" ht="16.5" thickBot="1">
       <c r="A112" s="4">
         <v>111</v>
       </c>
@@ -3076,7 +3070,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="113" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" ht="16.5" thickBot="1">
       <c r="A113" s="4">
         <v>112</v>
       </c>
@@ -3092,7 +3086,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="114" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" ht="16.5" thickBot="1">
       <c r="A114" s="4">
         <v>113</v>
       </c>
@@ -3108,7 +3102,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="115" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" ht="16.5" thickBot="1">
       <c r="A115" s="4">
         <v>114</v>
       </c>
@@ -3124,7 +3118,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="116" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" ht="16.5" thickBot="1">
       <c r="A116" s="4">
         <v>115</v>
       </c>
@@ -3140,7 +3134,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="117" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" ht="16.5" thickBot="1">
       <c r="A117" s="4">
         <v>116</v>
       </c>
@@ -3156,7 +3150,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="118" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" ht="16.5" thickBot="1">
       <c r="A118" s="4">
         <v>117</v>
       </c>
@@ -3172,7 +3166,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="119" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" ht="16.5" thickBot="1">
       <c r="A119" s="4">
         <v>118</v>
       </c>
@@ -3188,7 +3182,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="120" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" ht="16.5" thickBot="1">
       <c r="A120" s="4">
         <v>119</v>
       </c>
@@ -3204,7 +3198,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="121" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" ht="16.5" thickBot="1">
       <c r="A121" s="4">
         <v>120</v>
       </c>
@@ -3220,7 +3214,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="122" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" ht="16.5" thickBot="1">
       <c r="A122" s="4">
         <v>121</v>
       </c>
@@ -3236,7 +3230,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="123" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" ht="16.5" thickBot="1">
       <c r="A123" s="4">
         <v>122</v>
       </c>
@@ -3252,7 +3246,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="124" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" ht="16.5" thickBot="1">
       <c r="A124" s="4">
         <v>123</v>
       </c>
@@ -3268,7 +3262,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="125" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" ht="16.5" thickBot="1">
       <c r="A125" s="4">
         <v>124</v>
       </c>
@@ -3284,7 +3278,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="126" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" ht="16.5" thickBot="1">
       <c r="A126" s="4">
         <v>125</v>
       </c>
@@ -3300,7 +3294,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="127" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" ht="16.5" thickBot="1">
       <c r="A127" s="4">
         <v>126</v>
       </c>
@@ -3316,7 +3310,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="128" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" ht="16.5" thickBot="1">
       <c r="A128" s="4">
         <v>127</v>
       </c>
@@ -3332,7 +3326,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="129" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" ht="16.5" thickBot="1">
       <c r="A129" s="4">
         <v>128</v>
       </c>
@@ -3348,7 +3342,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="130" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" ht="16.5" thickBot="1">
       <c r="A130" s="4">
         <v>129</v>
       </c>
@@ -3364,7 +3358,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="131" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" ht="16.5" thickBot="1">
       <c r="A131" s="4">
         <v>130</v>
       </c>
@@ -3380,7 +3374,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="132" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" ht="16.5" thickBot="1">
       <c r="A132" s="4">
         <v>131</v>
       </c>
@@ -3396,7 +3390,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="133" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" ht="16.5" thickBot="1">
       <c r="A133" s="4">
         <v>132</v>
       </c>
@@ -3412,7 +3406,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="134" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" ht="16.5" thickBot="1">
       <c r="A134" s="4">
         <v>133</v>
       </c>
@@ -3428,7 +3422,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="135" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" ht="16.5" thickBot="1">
       <c r="A135" s="4">
         <v>134</v>
       </c>
@@ -3444,7 +3438,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="136" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" ht="16.5" thickBot="1">
       <c r="A136" s="4">
         <v>135</v>
       </c>
@@ -3460,7 +3454,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="137" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" ht="16.5" thickBot="1">
       <c r="A137" s="4">
         <v>136</v>
       </c>
@@ -3476,7 +3470,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="138" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" ht="16.5" thickBot="1">
       <c r="A138" s="4">
         <v>137</v>
       </c>
@@ -3492,7 +3486,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="139" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" ht="16.5" thickBot="1">
       <c r="A139" s="4">
         <v>138</v>
       </c>
@@ -3508,7 +3502,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="140" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" ht="16.5" thickBot="1">
       <c r="A140" s="4">
         <v>139</v>
       </c>
@@ -3524,7 +3518,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="141" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" ht="16.5" thickBot="1">
       <c r="A141" s="4">
         <v>140</v>
       </c>
@@ -3540,7 +3534,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="142" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" ht="16.5" thickBot="1">
       <c r="A142" s="4">
         <v>141</v>
       </c>
@@ -3556,7 +3550,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="143" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" ht="16.5" thickBot="1">
       <c r="A143" s="4">
         <v>142</v>
       </c>
@@ -3572,7 +3566,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="144" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" ht="16.5" thickBot="1">
       <c r="A144" s="4">
         <v>143</v>
       </c>
@@ -3588,7 +3582,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="145" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" ht="16.5" thickBot="1">
       <c r="A145" s="4">
         <v>144</v>
       </c>
@@ -3604,7 +3598,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="146" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" ht="16.5" thickBot="1">
       <c r="A146" s="4">
         <v>145</v>
       </c>
@@ -3620,7 +3614,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="147" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" ht="16.5" thickBot="1">
       <c r="A147" s="4">
         <v>146</v>
       </c>
@@ -3636,7 +3630,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="148" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" ht="16.5" thickBot="1">
       <c r="A148" s="4">
         <v>147</v>
       </c>
@@ -3652,7 +3646,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="149" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" ht="16.5" thickBot="1">
       <c r="A149" s="4">
         <v>148</v>
       </c>
@@ -3668,7 +3662,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="150" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" ht="16.5" thickBot="1">
       <c r="A150" s="4">
         <v>149</v>
       </c>
@@ -3684,7 +3678,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="151" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" ht="16.5" thickBot="1">
       <c r="A151" s="4">
         <v>150</v>
       </c>
@@ -3700,7 +3694,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="152" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" ht="16.5" thickBot="1">
       <c r="A152" s="4">
         <v>151</v>
       </c>
@@ -3716,7 +3710,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="153" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" ht="16.5" thickBot="1">
       <c r="A153" s="4">
         <v>152</v>
       </c>
@@ -3732,7 +3726,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="154" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5" ht="16.5" thickBot="1">
       <c r="A154" s="4">
         <v>153</v>
       </c>
@@ -3748,7 +3742,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="155" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5" ht="16.5" thickBot="1">
       <c r="A155" s="4">
         <v>154</v>
       </c>
@@ -3764,7 +3758,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="156" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5" ht="16.5" thickBot="1">
       <c r="A156" s="4">
         <v>155</v>
       </c>
@@ -3780,7 +3774,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="157" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5" ht="16.5" thickBot="1">
       <c r="A157" s="4">
         <v>156</v>
       </c>
@@ -3796,7 +3790,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="158" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:5" ht="16.5" thickBot="1">
       <c r="A158" s="4">
         <v>157</v>
       </c>
@@ -3812,7 +3806,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="159" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5" ht="16.5" thickBot="1">
       <c r="A159" s="4">
         <v>158</v>
       </c>
@@ -3828,7 +3822,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="160" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5" ht="16.5" thickBot="1">
       <c r="A160" s="4">
         <v>159</v>
       </c>
@@ -3844,7 +3838,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="161" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5" ht="16.5" thickBot="1">
       <c r="A161" s="4">
         <v>160</v>
       </c>
@@ -3860,7 +3854,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="162" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5" ht="16.5" thickBot="1">
       <c r="A162" s="4">
         <v>161</v>
       </c>
@@ -3876,7 +3870,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="163" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5" ht="16.5" thickBot="1">
       <c r="A163" s="4">
         <v>162</v>
       </c>
@@ -3892,7 +3886,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="164" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5" ht="16.5" thickBot="1">
       <c r="A164" s="4">
         <v>163</v>
       </c>
@@ -3908,7 +3902,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="165" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5" ht="16.5" thickBot="1">
       <c r="A165" s="4">
         <v>164</v>
       </c>
@@ -3924,7 +3918,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="166" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5" ht="16.5" thickBot="1">
       <c r="A166" s="4">
         <v>165</v>
       </c>
@@ -3940,7 +3934,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="167" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5" ht="16.5" thickBot="1">
       <c r="A167" s="4">
         <v>166</v>
       </c>
@@ -3956,7 +3950,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="168" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5" ht="16.5" thickBot="1">
       <c r="A168" s="4">
         <v>167</v>
       </c>
@@ -3972,7 +3966,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="169" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5" ht="16.5" thickBot="1">
       <c r="A169" s="4">
         <v>168</v>
       </c>
@@ -3988,7 +3982,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="170" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5" ht="16.5" thickBot="1">
       <c r="A170" s="4">
         <v>169</v>
       </c>
@@ -4004,7 +3998,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="171" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" ht="16.5" thickBot="1">
       <c r="A171" s="4">
         <v>170</v>
       </c>
@@ -4020,7 +4014,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="172" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5" ht="16.5" thickBot="1">
       <c r="A172" s="4">
         <v>171</v>
       </c>
@@ -4036,7 +4030,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="173" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5" ht="16.5" thickBot="1">
       <c r="A173" s="4">
         <v>172</v>
       </c>
@@ -4052,7 +4046,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="174" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" ht="16.5" thickBot="1">
       <c r="A174" s="4">
         <v>173</v>
       </c>
@@ -4068,7 +4062,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="175" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" ht="16.5" thickBot="1">
       <c r="A175" s="4">
         <v>174</v>
       </c>
@@ -4084,7 +4078,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="176" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" ht="16.5" thickBot="1">
       <c r="A176" s="4">
         <v>175</v>
       </c>
@@ -4100,7 +4094,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="177" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" ht="16.5" thickBot="1">
       <c r="A177" s="4">
         <v>176</v>
       </c>
@@ -4116,7 +4110,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="178" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" ht="16.5" thickBot="1">
       <c r="A178" s="4">
         <v>177</v>
       </c>
@@ -4132,7 +4126,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="179" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" ht="16.5" thickBot="1">
       <c r="A179" s="4">
         <v>178</v>
       </c>
@@ -4148,7 +4142,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="180" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" ht="16.5" thickBot="1">
       <c r="A180" s="4">
         <v>179</v>
       </c>
@@ -4164,7 +4158,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="181" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" ht="16.5" thickBot="1">
       <c r="A181" s="4">
         <v>180</v>
       </c>
@@ -4180,7 +4174,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="182" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" ht="16.5" thickBot="1">
       <c r="A182" s="4">
         <v>181</v>
       </c>
@@ -4196,7 +4190,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="183" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" ht="16.5" thickBot="1">
       <c r="A183" s="4">
         <v>182</v>
       </c>
@@ -4212,7 +4206,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="184" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" ht="16.5" thickBot="1">
       <c r="A184" s="4">
         <v>183</v>
       </c>
@@ -4228,7 +4222,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="185" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" ht="16.5" thickBot="1">
       <c r="A185" s="4">
         <v>184</v>
       </c>
@@ -4244,7 +4238,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="186" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" ht="16.5" thickBot="1">
       <c r="A186" s="4">
         <v>185</v>
       </c>
@@ -4260,7 +4254,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="187" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" ht="16.5" thickBot="1">
       <c r="A187" s="4">
         <v>186</v>
       </c>
@@ -4276,7 +4270,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="188" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:5" ht="16.5" thickBot="1">
       <c r="A188" s="4">
         <v>187</v>
       </c>
@@ -4292,7 +4286,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="189" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:5" ht="16.5" thickBot="1">
       <c r="A189" s="4">
         <v>188</v>
       </c>
@@ -4308,7 +4302,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="190" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:5" ht="16.5" thickBot="1">
       <c r="A190" s="4">
         <v>189</v>
       </c>
@@ -4324,7 +4318,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="191" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:5" ht="16.5" thickBot="1">
       <c r="A191" s="4">
         <v>190</v>
       </c>
@@ -4340,7 +4334,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="192" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:5" ht="16.5" thickBot="1">
       <c r="A192" s="4">
         <v>191</v>
       </c>
@@ -4356,7 +4350,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="193" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:5" ht="16.5" thickBot="1">
       <c r="A193" s="4">
         <v>192</v>
       </c>
@@ -4372,7 +4366,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="194" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:5" ht="16.5" thickBot="1">
       <c r="A194" s="4">
         <v>193</v>
       </c>
@@ -4388,7 +4382,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="195" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:5" ht="16.5" thickBot="1">
       <c r="A195" s="4">
         <v>194</v>
       </c>
@@ -4404,7 +4398,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="196" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:5" ht="16.5" thickBot="1">
       <c r="A196" s="4">
         <v>195</v>
       </c>
@@ -4420,7 +4414,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="197" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:5" ht="16.5" thickBot="1">
       <c r="A197" s="4">
         <v>196</v>
       </c>
@@ -4436,7 +4430,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="198" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:5" ht="16.5" thickBot="1">
       <c r="A198" s="4">
         <v>197</v>
       </c>
@@ -4452,7 +4446,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="199" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:5" ht="16.5" thickBot="1">
       <c r="A199" s="4">
         <v>198</v>
       </c>
@@ -4468,7 +4462,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="200" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:5" ht="16.5" thickBot="1">
       <c r="A200" s="4">
         <v>199</v>
       </c>
@@ -4484,7 +4478,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="201" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:5" ht="16.5" thickBot="1">
       <c r="A201" s="4">
         <v>200</v>
       </c>
@@ -4500,7 +4494,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="202" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:5" ht="16.5" thickBot="1">
       <c r="A202" s="4">
         <v>201</v>
       </c>
@@ -4516,7 +4510,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="203" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:5" ht="16.5" thickBot="1">
       <c r="A203" s="4">
         <v>202</v>
       </c>
@@ -4532,7 +4526,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="204" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:5" ht="16.5" thickBot="1">
       <c r="A204" s="4">
         <v>203</v>
       </c>
@@ -4548,7 +4542,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="205" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:5" ht="16.5" thickBot="1">
       <c r="A205" s="4">
         <v>204</v>
       </c>
@@ -4564,7 +4558,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="206" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:5" ht="16.5" thickBot="1">
       <c r="A206" s="4">
         <v>205</v>
       </c>
@@ -4580,7 +4574,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="207" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:5" ht="16.5" thickBot="1">
       <c r="A207" s="4">
         <v>206</v>
       </c>
@@ -4596,7 +4590,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="208" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:5" ht="16.5" thickBot="1">
       <c r="A208" s="4">
         <v>207</v>
       </c>
@@ -4612,7 +4606,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="209" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:5" ht="16.5" thickBot="1">
       <c r="A209" s="4">
         <v>208</v>
       </c>
@@ -4628,7 +4622,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="210" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:5" ht="16.5" thickBot="1">
       <c r="A210" s="4">
         <v>209</v>
       </c>
@@ -4644,7 +4638,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="211" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:5" ht="16.5" thickBot="1">
       <c r="A211" s="4">
         <v>210</v>
       </c>
@@ -4660,7 +4654,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="212" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:5" ht="16.5" thickBot="1">
       <c r="A212" s="4">
         <v>211</v>
       </c>
@@ -4676,7 +4670,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="213" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:5" ht="16.5" thickBot="1">
       <c r="A213" s="4">
         <v>212</v>
       </c>
@@ -4692,7 +4686,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="214" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:5" ht="16.5" thickBot="1">
       <c r="A214" s="4">
         <v>213</v>
       </c>
@@ -4708,7 +4702,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="215" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:5" ht="16.5" thickBot="1">
       <c r="A215" s="4">
         <v>214</v>
       </c>
@@ -4724,7 +4718,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="216" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:5" ht="16.5" thickBot="1">
       <c r="A216" s="4">
         <v>215</v>
       </c>
@@ -4740,7 +4734,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="217" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:5" ht="16.5" thickBot="1">
       <c r="A217" s="4">
         <v>216</v>
       </c>
@@ -4756,7 +4750,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="218" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:5" ht="16.5" thickBot="1">
       <c r="A218" s="4">
         <v>217</v>
       </c>
@@ -4772,7 +4766,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="219" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:5" ht="16.5" thickBot="1">
       <c r="A219" s="4">
         <v>218</v>
       </c>
@@ -4788,7 +4782,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="220" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:5" ht="16.5" thickBot="1">
       <c r="A220" s="4">
         <v>219</v>
       </c>
@@ -4804,7 +4798,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="221" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:5" ht="16.5" thickBot="1">
       <c r="A221" s="4">
         <v>220</v>
       </c>
@@ -4820,7 +4814,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="222" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:5" ht="16.5" thickBot="1">
       <c r="A222" s="4">
         <v>221</v>
       </c>
@@ -4836,7 +4830,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="223" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:5" ht="16.5" thickBot="1">
       <c r="A223" s="4">
         <v>222</v>
       </c>
@@ -4852,7 +4846,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="224" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:5" ht="16.5" thickBot="1">
       <c r="A224" s="4">
         <v>223</v>
       </c>
@@ -4868,7 +4862,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="225" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:5" ht="16.5" thickBot="1">
       <c r="A225" s="4">
         <v>224</v>
       </c>
@@ -4884,7 +4878,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="226" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:5" ht="16.5" thickBot="1">
       <c r="A226" s="4">
         <v>225</v>
       </c>
@@ -4900,7 +4894,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="227" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:5" ht="16.5" thickBot="1">
       <c r="A227" s="4">
         <v>226</v>
       </c>
@@ -4916,7 +4910,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="228" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:5" ht="16.5" thickBot="1">
       <c r="A228" s="4">
         <v>227</v>
       </c>
@@ -4932,7 +4926,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="229" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:5" ht="16.5" thickBot="1">
       <c r="A229" s="4">
         <v>228</v>
       </c>
@@ -4948,7 +4942,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="230" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:5" ht="16.5" thickBot="1">
       <c r="A230" s="4">
         <v>229</v>
       </c>
@@ -4964,7 +4958,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="231" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:5" ht="16.5" thickBot="1">
       <c r="A231" s="4">
         <v>230</v>
       </c>
@@ -4980,7 +4974,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="232" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:5" ht="16.5" thickBot="1">
       <c r="A232" s="4">
         <v>231</v>
       </c>
@@ -4996,7 +4990,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="233" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:5" ht="16.5" thickBot="1">
       <c r="A233" s="4">
         <v>232</v>
       </c>
@@ -5012,7 +5006,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="234" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:5" ht="16.5" thickBot="1">
       <c r="A234" s="4">
         <v>233</v>
       </c>
@@ -5028,7 +5022,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="235" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:5" ht="16.5" thickBot="1">
       <c r="A235" s="4">
         <v>234</v>
       </c>
@@ -5044,7 +5038,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="236" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:5" ht="16.5" thickBot="1">
       <c r="A236" s="4">
         <v>235</v>
       </c>
@@ -5060,7 +5054,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="237" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:5" ht="16.5" thickBot="1">
       <c r="A237" s="4">
         <v>236</v>
       </c>
@@ -5076,7 +5070,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="238" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:5" ht="16.5" thickBot="1">
       <c r="A238" s="4">
         <v>237</v>
       </c>
@@ -5092,7 +5086,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="239" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:5" ht="16.5" thickBot="1">
       <c r="A239" s="4">
         <v>238</v>
       </c>
@@ -5108,7 +5102,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="240" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:5" ht="16.5" thickBot="1">
       <c r="A240" s="4">
         <v>239</v>
       </c>
@@ -5124,7 +5118,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="241" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:5" ht="16.5" thickBot="1">
       <c r="A241" s="4">
         <v>240</v>
       </c>
@@ -5140,7 +5134,7 @@
         <v xml:space="preserve">Decimal </v>
       </c>
     </row>
-    <row r="242" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:5" ht="16.5" thickBot="1">
       <c r="A242" s="4">
         <v>241</v>
       </c>
@@ -5156,7 +5150,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="243" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:5" ht="16.5" thickBot="1">
       <c r="A243" s="4">
         <v>242</v>
       </c>
@@ -5172,7 +5166,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="244" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:5" ht="16.5" thickBot="1">
       <c r="A244" s="4">
         <v>243</v>
       </c>
@@ -5188,7 +5182,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="245" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:5" ht="16.5" thickBot="1">
       <c r="A245" s="4">
         <v>244</v>
       </c>
@@ -5204,7 +5198,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="246" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:5" ht="16.5" thickBot="1">
       <c r="A246" s="4">
         <v>245</v>
       </c>
@@ -5220,7 +5214,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="247" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:5" ht="16.5" thickBot="1">
       <c r="A247" s="4">
         <v>246</v>
       </c>
@@ -5236,7 +5230,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="248" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:5" ht="16.5" thickBot="1">
       <c r="A248" s="4">
         <v>247</v>
       </c>
@@ -5252,7 +5246,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="249" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:5" ht="16.5" thickBot="1">
       <c r="A249" s="4">
         <v>248</v>
       </c>
@@ -5268,7 +5262,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="250" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:5" ht="16.5" thickBot="1">
       <c r="A250" s="4">
         <v>249</v>
       </c>
@@ -5284,7 +5278,7 @@
         <v xml:space="preserve">Char </v>
       </c>
     </row>
-    <row r="251" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:5" ht="16.5" thickBot="1">
       <c r="A251" s="4">
         <v>250</v>
       </c>

</xml_diff>